<commit_message>
fix(imagenes): corregir persistencia de fotos en Cloudinary
</commit_message>
<xml_diff>
--- a/backend/prueba_reporte_refugio.xlsx
+++ b/backend/prueba_reporte_refugio.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Historial de Solicitudes del Re" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historial de Solicitudes del Re'!$A$4:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Historial de Solicitudes del Re'!$A$4:$H$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Historial de Solicitudes del Re'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -205,6 +205,36 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="933450" cy="495300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -494,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -507,17 +537,17 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Historial de Solicitudes del Refugio</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generado el 21/08/2026 01:37 (UTC) · patitas · Adoptify</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Generado el 23/08/2026 01:13 (UTC) · patitas · Adoptify</t>
         </is>
       </c>
     </row>
@@ -565,31 +595,31 @@
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Alexandra Hernandez</t>
+          <t>Kevin Donoso</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>ah0177351@gmail.com</t>
+          <t>kdonoso12376@gmail.com</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>3134655122</t>
+          <t>3184050242</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Kika</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -598,54 +628,93 @@
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>46248.81326510105</v>
+        <v>46255.85923367919</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Alexandra Hernandez</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>ah0177351@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>3134655122</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Kika</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>46248.81326510105</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>ALISSON</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>alissonflorezaroca@gmail.com</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>312020201</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>muñeca</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H7" s="7" t="n">
         <v>46243.12075571842</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H6"/>
+  <autoFilter ref="A4:H7"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>